<commit_message>
test: make fixture branches live, add select_multiple, repeat_count, drift guards
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/tests/fixtures/amb_asha_visit.xlsx
+++ b/server/tests/fixtures/amb_asha_visit.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,6 +489,11 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>repeat_count</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -712,6 +717,11 @@
           <t>Children roster</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>${household_children}</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -852,183 +862,254 @@
           <t>Which IFA does the child receive?</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>${child_age_months} &gt;= 6</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>select_one yes_no</t>
+          <t>select_multiple symptom</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>syrup_given</t>
+          <t>symptoms</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>क्या बच्चे को आई एफ ए सिरप पिलाया गया?</t>
+          <t>इस दौरे में बच्चे में कौन से लक्षण दिखे?</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Was the child given IFA syrup?</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>${ifa_form} = 'syrup'</t>
+          <t>Which symptoms were seen during this visit?</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>begin repeat</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ifa_doses</t>
+          <t>referral_note</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>आई एफ ए खुराक का रिकॉर्ड</t>
+          <t>स्वास्थ्य केंद्र भेजने की वजह लिखें</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IFA dose record</t>
+          <t>Write the reason for referral</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>${syrup_given} = 'yes'</t>
+          <t>selected(${symptoms}, 'pallor')</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>dose_date</t>
+          <t>tablet_taken</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>खुराक की तारीख</t>
+          <t>क्या बच्चे ने इस हफ़्ते गोली खाई?</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Dose date</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>तारीख आज से आगे की नहीं हो सकती</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>The date cannot be in the future</t>
+          <t>Did the child take the tablet this week?</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>${ifa_form} != 'syrup' and ${child_age_years} &gt;= 3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one yes_no</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>dose_ml</t>
+          <t>syrup_given</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>खुराक (मिलीलीटर)</t>
+          <t>क्या बच्चे को आई एफ ए सिरप पिलाया गया?</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Dose (ml)</t>
+          <t>Was the child given IFA syrup?</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>${ifa_form} = 'syrup'</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>end repeat</t>
+          <t>begin repeat</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ifa_doses</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>आई एफ ए खुराक का रिकॉर्ड</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IFA dose record</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>${syrup_given} = 'yes'</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>end repeat</t>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>dose_date</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>खुराक की तारीख</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Dose date</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>. &lt;= today()</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>तारीख आज से आगे की नहीं हो सकती</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>The date cannot be in the future</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>children_count</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>count(${child_name})</t>
+          <t>dose_ml</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>खुराक (मिलीलीटर)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Dose (ml)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>end repeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>end repeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>children_count</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>count(${child_name})</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>summary_note</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>धन्यवाद, यह दौरा पूरा हुआ</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Thank you, visit complete</t>
         </is>
@@ -1045,7 +1126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1438,20 +1519,108 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>symptom</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>pallor</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>हथेली या आँखें पीली</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pale palms or eyes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>symptom</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>fatigue</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>जल्दी थक जाता है</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tires easily</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>symptom</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>breathless</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>साँस फूलना</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Breathlessness</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>symptom</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>कोई लक्षण नहीं</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>No symptoms</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>ifa_form</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>blue</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>आई एफ ए नीली गोली</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>IFA blue tablet</t>
         </is>

</xml_diff>